<commit_message>
Polish LENA report: real Figma icons, fixed TOC, exact contact-panel style
- Swapped the hand-drawn placeholder icons for the actual Material icons
  exported from the Figma design (child info, stat cards, section
  headings, category headings, TOC "clickable report" hint, and the
  phone/email/link/address icons in every resource-directory contact
  panel), matching the design's colors (dark icons, #CA732B accent for
  contact rows) instead of guessed ones.
- Fixed two wrong icon reuses on page 6: "Participants" and "Collection
  Context" were reusing unrelated icons; now use the correct people/home
  icons.
- Added two TOC entries the first pass missed (LENA Result, Important
  Note under Overview) with matching in-page anchors.
- Stripped the alpha-mask wrapper Figma's export includes on every icon —
  WeasyPrint doesn't fully honor it, which showed up as a stray gray
  bounding box behind the category-heading icon.
</commit_message>
<xml_diff>
--- a/report_types/lena/translations.xlsx
+++ b/report_types/lena/translations.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B265"/>
+  <dimension ref="A1:B266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2063,1546 +2063,1558 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>LENA Results</t>
+          <t>LENA Result</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Resultados de LENA</t>
+          <t>Resultado LENA</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>LENA automatically detects speech in both English and Spanish, words in both languages are counted by LENA.</t>
+          <t>LENA Results</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>LENA detecta automáticamente el habla tanto en inglés como en español, LENA cuenta las palabras en ambos idiomas.</t>
+          <t>Resultados de LENA</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>LENA measured the natural audio environment of your child and categorized the different types of sounds that your child could hear, and for how long they were exposed to each one.</t>
+          <t>LENA automatically detects speech in both English and Spanish, words in both languages are counted by LENA.</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>LENA midió el entorno auditivo natural de su hijo y clasificó los diferentes tipos de sonidos que su hijo podía escuchar y durante cuánto tiempo estuvo expuesto a cada uno.</t>
+          <t>LENA detecta automáticamente el habla tanto en inglés como en español, LENA cuenta las palabras en ambos idiomas.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Lantern</t>
+          <t>LENA measured the natural audio environment of your child and categorized the different types of sounds that your child could hear, and for how long they were exposed to each one.</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Linterna</t>
+          <t>LENA midió el entorno auditivo natural de su hijo y clasificó los diferentes tipos de sonidos que su hijo podía escuchar y durante cuánto tiempo estuvo expuesto a cada uno.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Lantern is a national nonprofit dedicated to providing families with essential information for raising kids, from pregnancy through the preteen years.</t>
+          <t>Lantern</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Lantern es una organización nacional sin fines de lucro dedicada a brindar a las familias información esencial para la crianza de sus hijos, desde el embarazo hasta la preadolescencia.</t>
+          <t>Linterna</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Learn About Your Report</t>
+          <t>Lantern is a national nonprofit dedicated to providing families with essential information for raising kids, from pregnancy through the preteen years.</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Obtenga más información sobre su informe</t>
+          <t>Lantern es una organización nacional sin fines de lucro dedicada a brindar a las familias información esencial para la crianza de sus hijos, desde el embarazo hasta la preadolescencia.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Least Productivity</t>
+          <t>Learn About Your Report</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Menos productividad</t>
+          <t>Obtenga más información sobre su informe</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Least Turns</t>
+          <t>Least Productivity</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Menos vueltas</t>
+          <t>Menos productividad</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Least Vocalizations</t>
+          <t>Least Turns</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Menos vocalizaciones</t>
+          <t>Menos vueltas</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Lena report</t>
+          <t>Least Vocalizations</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>informe lena</t>
+          <t>Menos vocalizaciones</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Lirios Pediatrics</t>
+          <t>Lena report</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Pediatría Lirios</t>
+          <t>informe lena</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Low (1-24)</t>
+          <t>Lirios Pediatrics</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Bajo (1-24)</t>
+          <t>Pediatría Lirios</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Low Average (25-49)</t>
+          <t>Low (1-24)</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Promedio bajo (25-49)</t>
+          <t>Bajo (1-24)</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>MIOP's team consists of DSHS Certified Community Health Workers (CHWs) with direct lived experience who provide psychosocial support to Black and African American women in Travis County.</t>
+          <t>Low Average (25-49)</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>El equipo de MIOP está formado por trabajadores de salud comunitarios (CHW) certificados por DSHS con experiencia vivida directamente que brindan apoyo psicosocial a mujeres negras y afroamericanas en el condado de Travis.</t>
+          <t>Promedio bajo (25-49)</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Make faces, use gestures</t>
+          <t>MIOP's team consists of DSHS Certified Community Health Workers (CHWs) with direct lived experience who provide psychosocial support to Black and African American women in Travis County.</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Haz muecas, usa gestos.</t>
+          <t>El equipo de MIOP está formado por trabajadores de salud comunitarios (CHW) certificados por DSHS con experiencia vivida directamente que brindan apoyo psicosocial a mujeres negras y afroamericanas en el condado de Travis.</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Maternal Infant Outreach Program (MIOP)</t>
+          <t>Make faces, use gestures</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Programa de extensión maternoinfantil (MIOP)</t>
+          <t>Haz muecas, usa gestos.</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Mobile Clinic in Creedmoor</t>
+          <t>Maternal Infant Outreach Program (MIOP)</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Clínica móvil en Creedmoor</t>
+          <t>Programa de extensión maternoinfantil (MIOP)</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Most Active Time: 05:00-06:00 PM</t>
+          <t>Mobile Clinic in Creedmoor</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Hora más activa: 05:00-06:00 p.m.</t>
+          <t>Clínica móvil en Creedmoor</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Most Active Time: 06:00-07:00 PM</t>
+          <t>Most Active Time: 05:00-06:00 PM</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Hora más activa: 06:00-07:00 p.m.</t>
+          <t>Hora más activa: 05:00-06:00 p.m.</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Most Active Time: 08:00-09:00 AM</t>
+          <t>Most Active Time: 06:00-07:00 PM</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Hora más activa: 08:00-09:00 a. m.</t>
+          <t>Hora más activa: 06:00-07:00 p.m.</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Most Productivity</t>
+          <t>Most Active Time: 08:00-09:00 AM</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Mayor productividad</t>
+          <t>Hora más activa: 08:00-09:00 a. m.</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Most Turns</t>
+          <t>Most Productivity</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>La mayoría de los turnos</t>
+          <t>Mayor productividad</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Most Vocalizations</t>
+          <t>Most Turns</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>La mayoría de las vocalizaciones</t>
+          <t>La mayoría de los turnos</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Name things</t>
+          <t>Most Vocalizations</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Nombrar cosas</t>
+          <t>La mayoría de las vocalizaciones</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Newborn &amp; maternal health screenings</t>
+          <t>Name things</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Exámenes de salud materna y neonatal</t>
+          <t>Nombrar cosas</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Noise</t>
+          <t>Newborn &amp; maternal health screenings</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Ruido</t>
+          <t>Exámenes de salud materna y neonatal</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Offer walk-in primary care, behavioral health, dental, women's health, and pharmacy services to uninsured/under-insured residents of Travis County.</t>
+          <t>Noise</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Ofrecer servicios de atención primaria, salud conductual, dental, salud de la mujer y farmacia sin cita previa a residentes sin seguro o con seguro insuficiente del condado de Travis.</t>
+          <t>Ruido</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Offers financial assistance &amp; sliding fee scale</t>
+          <t>Offer walk-in primary care, behavioral health, dental, women's health, and pharmacy services to uninsured/under-insured residents of Travis County.</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Ofrece asistencia financiera y escala móvil de tarifas</t>
+          <t>Ofrecer servicios de atención primaria, salud conductual, dental, salud de la mujer y farmacia sin cita previa a residentes sin seguro o con seguro insuficiente del condado de Travis.</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Overlap</t>
+          <t>Offers financial assistance &amp; sliding fee scale</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Superposición</t>
+          <t>Ofrece asistencia financiera y escala móvil de tarifas</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>Overlap</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Descripción general</t>
+          <t>Superposición</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Parent-child class</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>clase de padres e hijos</t>
+          <t>Descripción general</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Parenting</t>
+          <t>Parent-child class</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Crianza de los hijos</t>
+          <t>clase de padres e hijos</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Parenting Classes &amp; Support</t>
+          <t>Parenting</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Clases y apoyo para padres</t>
+          <t>Crianza de los hijos</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Parenting classes &amp; abortion healing support</t>
+          <t>Parenting Classes &amp; Support</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Clases para padres y apoyo para la curación del aborto</t>
+          <t>Clases y apoyo para padres</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Participants: 329 children</t>
+          <t>Parenting classes &amp; abortion healing support</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Participantes: 329 niños</t>
+          <t>Clases para padres y apoyo para la curación del aborto</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Peer support for Black and African American women</t>
+          <t>Participants: 329 children</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Apoyo entre pares para mujeres negras y afroamericanas</t>
+          <t>Participantes: 329 niños</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Percentile Key: High</t>
+          <t>Peer support for Black and African American women</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Clave de percentil: alta</t>
+          <t>Apoyo entre pares para mujeres negras y afroamericanas</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Percentile Key: High Average</t>
+          <t>Percentile Key: High</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Clave de percentil: promedio alto</t>
+          <t>Clave de percentil: alta</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Percentile Key: Low Average</t>
+          <t>Percentile Key: High Average</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Clave de percentil: promedio bajo</t>
+          <t>Clave de percentil: promedio alto</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Percentiles Key</t>
+          <t>Percentile Key: Low Average</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Clave de percentiles</t>
+          <t>Clave de percentil: promedio bajo</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Percentiles compare your results to other parents and children who have used LENA.</t>
+          <t>Percentiles Key</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Los percentiles comparan sus resultados con los de otros padres y niños que han usado LENA.</t>
+          <t>Clave de percentiles</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Produced by WCWH</t>
+          <t>Percentiles compare your results to other parents and children who have used LENA.</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Producido por WCWH</t>
+          <t>Los percentiles comparan sus resultados con los de otros padres y niños que han usado LENA.</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Programs and services to help families and new moms build stability, develop skills, and reach their full potential.</t>
+          <t>Produced by WCWH</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Programas y servicios para ayudar a las familias y a las nuevas mamás a generar estabilidad, desarrollar habilidades y alcanzar su máximo potencial.</t>
+          <t>Producido por WCWH</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Provide all primary care services for child, including well checks, care for illness and injury, care for chronic problems, and hospital follow-up.</t>
+          <t>Programs and services to help families and new moms build stability, develop skills, and reach their full potential.</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Proporcionar todos los servicios de atención primaria para niños, incluidos controles de bienestar, atención de enfermedades y lesiones, atención de problemas crónicos y seguimiento hospitalario.</t>
+          <t>Programas y servicios para ayudar a las familias y a las nuevas mamás a generar estabilidad, desarrollar habilidades y alcanzar su máximo potencial.</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Provide children and their families access to books and resources to support the development of early literacy skills and foster a love of reading.</t>
+          <t>Provide all primary care services for child, including well checks, care for illness and injury, care for chronic problems, and hospital follow-up.</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Brindar a los niños y sus familias acceso a libros y recursos para apoyar el desarrollo de habilidades de alfabetización temprana y fomentar el amor por la lectura.</t>
+          <t>Proporcionar todos los servicios de atención primaria para niños, incluidos controles de bienestar, atención de enfermedades y lesiones, atención de problemas crónicos y seguimiento hospitalario.</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Provide quality healthcare and various medical, dental, and mental health.</t>
+          <t>Provide children and their families access to books and resources to support the development of early literacy skills and foster a love of reading.</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Brindar atención médica de calidad y diversos servicios médicos, dentales y de salud mental.</t>
+          <t>Brindar a los niños y sus familias acceso a libros y recursos para apoyar el desarrollo de habilidades de alfabetización temprana y fomentar el amor por la lectura.</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Questions and Concerns</t>
+          <t>Provide quality healthcare and various medical, dental, and mental health.</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Preguntas e inquietudes</t>
+          <t>Brindar atención médica de calidad y diversos servicios médicos, dentales y de salud mental.</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Recording Hours: 32,000+ hours</t>
+          <t>Questions and Concerns</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Horas de grabación: más de 32.000 horas</t>
+          <t>Preguntas e inquietudes</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Register Here</t>
+          <t>Recording Hours: 32,000+ hours</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Regístrese aquí</t>
+          <t>Horas de grabación: más de 32.000 horas</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Relative Score: 45th percentile</t>
+          <t>Register Here</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Puntuación relativa: percentil 45</t>
+          <t>Regístrese aquí</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Relative Score: 60th percentile</t>
+          <t>Relative Score: 45th percentile</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Puntuación relativa: percentil 60</t>
+          <t>Puntuación relativa: percentil 45</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Relative Score: 82nd percentile</t>
+          <t>Relative Score: 60th percentile</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Puntuación relativa: percentil 82</t>
+          <t>Puntuación relativa: percentil 60</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Relative Score: 85th percentile</t>
+          <t>Relative Score: 82nd percentile</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Puntuación relativa: percentil 85</t>
+          <t>Puntuación relativa: percentil 82</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Relative Score: 90th percentile</t>
+          <t>Relative Score: 85th percentile</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Puntuación relativa: percentil 90</t>
+          <t>Puntuación relativa: percentil 85</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Relative Score: 95th percentile</t>
+          <t>Relative Score: 90th percentile</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Puntuación relativa: percentil 95</t>
+          <t>Puntuación relativa: percentil 90</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Relax and have fun!</t>
+          <t>Relative Score: 95th percentile</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>¡Relájate y diviértete!</t>
+          <t>Puntuación relativa: percentil 95</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Repeat and add</t>
+          <t>Relax and have fun!</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Repita y agregue</t>
+          <t>¡Relájate y diviértete!</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Research shows that when parents speak more to their children, it has positive effects on the child's vocabulary and language development.</t>
+          <t>Repeat and add</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Las investigaciones muestran que cuando los padres hablan más con sus hijos, esto tiene efectos positivos en el vocabulario y el desarrollo del lenguaje del niño.</t>
+          <t>Repita y agregue</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Resources</t>
+          <t>Research shows that when parents speak more to their children, it has positive effects on the child's vocabulary and language development.</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Recursos</t>
+          <t>Las investigaciones muestran que cuando los padres hablan más con sus hijos, esto tiene efectos positivos en el vocabulario y el desarrollo del lenguaje del niño.</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Results</t>
+          <t>Resources</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Resultados</t>
+          <t>Recursos</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Return to table of contents</t>
+          <t>Results</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Volver a la tabla de contenidos</t>
+          <t>Resultados</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Services by nurse practitioners &amp; students</t>
+          <t>Return to table of contents</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Servicios prestados por enfermeras practicantes y estudiantes.</t>
+          <t>Volver a la tabla de contenidos</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Session fee are based on income and household size</t>
+          <t>Services by nurse practitioners &amp; students</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>La tarifa de la sesión se basa en los ingresos y el tamaño del hogar.</t>
+          <t>Servicios prestados por enfermeras practicantes y estudiantes.</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Silence / Background</t>
+          <t>Session fee are based on income and household size</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Silencio / Fondo</t>
+          <t>La tarifa de la sesión se basa en los ingresos y el tamaño del hogar.</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Silence and very quiet/faint background sounds</t>
+          <t>Silence / Background</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Silencio y sonidos de fondo muy bajos/débiles.</t>
+          <t>Silencio / Fondo</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Sounds coming from a TV, speaker, or another electronic source</t>
+          <t>Silence and very quiet/faint background sounds</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Sonidos provenientes de un televisor, altavoz u otra fuente electrónica</t>
+          <t>Silencio y sonidos de fondo muy bajos/débiles.</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Speech</t>
+          <t>Sounds coming from a TV, speaker, or another electronic source</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Discurso</t>
+          <t>Sonidos provenientes de un televisor, altavoz u otra fuente electrónica</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Speech sounds and/or noises occurring at the same time</t>
+          <t>Speech</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Sonidos del habla y/o ruidos que ocurren al mismo tiempo.</t>
+          <t>Discurso</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Support Your Child's Language Growth</t>
+          <t>Speech sounds and/or noises occurring at the same time</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Apoye el crecimiento del lenguaje de su hijo</t>
+          <t>Sonidos del habla y/o ruidos que ocurren al mismo tiempo.</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Supports early brain development</t>
+          <t>Support Your Child's Language Growth</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Apoya el desarrollo temprano del cerebro.</t>
+          <t>Apoye el crecimiento del lenguaje de su hijo</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>TV/Electronic Sounds</t>
+          <t>Supports early brain development</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>TV/Sonidos electrónicos</t>
+          <t>Apoya el desarrollo temprano del cerebro.</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Table Of Contents</t>
+          <t>TV/Electronic Sounds</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Tabla de contenido</t>
+          <t>TV/Sonidos electrónicos</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Take turns</t>
+          <t>Table Of Contents</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Turnarse</t>
+          <t>Tabla de contenido</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Talk about</t>
+          <t>Take turns</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Hablar de</t>
+          <t>Turnarse</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Text (512) 593-1949</t>
+          <t>Talk about</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Texto (512) 593-1949</t>
+          <t>Hablar de</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>The LENA automatically detects speech in both English and Spanish, but the language and demographic makeup of the database can impact how well the results represent your child's experience.</t>
+          <t>Text (512) 593-1949</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>LENA detecta automáticamente el habla tanto en inglés como en español, pero el idioma y la composición demográfica de la base de datos pueden afectar la forma en que los resultados representan la experiencia de su hijo.</t>
+          <t>Texto (512) 593-1949</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>The LENA database is a group of 329 children's recordings collected by LENA to establish the norms for everyday language in young families.</t>
+          <t>The LENA automatically detects speech in both English and Spanish, but the language and demographic makeup of the database can impact how well the results represent your child's experience.</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>La base de datos LENA es un grupo de 329 grabaciones infantiles recopiladas por LENA para establecer las normas del lenguaje cotidiano en las familias jóvenes.</t>
+          <t>LENA detecta automáticamente el habla tanto en inglés como en español, pero el idioma y la composición demográfica de la base de datos pueden afectar la forma en que los resultados representan la experiencia de su hijo.</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>The LENA database mostly represents white (66%), English-speaking children from the US. Therefore, your percentiles may not fully reflect the norms for multilingual families or families of color.</t>
+          <t>The LENA database is a group of 329 children's recordings collected by LENA to establish the norms for everyday language in young families.</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>La base de datos de LENA representa principalmente a niños blancos (66%) de habla inglesa de Estados Unidos. Por lo tanto, es posible que sus percentiles no reflejen completamente las normas para familias multilingües o familias de color.</t>
+          <t>La base de datos LENA es un grupo de 329 grabaciones infantiles recopiladas por LENA para establecer las normas del lenguaje cotidiano en las familias jóvenes.</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>The different types of sound it measured include:</t>
+          <t>The LENA database mostly represents white (66%), English-speaking children from the US. Therefore, your percentiles may not fully reflect the norms for multilingual families or families of color.</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Los diferentes tipos de sonido que midió incluyen:</t>
+          <t>La base de datos de LENA representa principalmente a niños blancos (66%) de habla inglesa de Estados Unidos. Por lo tanto, es posible que sus percentiles no reflejen completamente las normas para familias multilingües o familias de color.</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>The length and variety of a child's speech while babbling or talking with an adult, reflecting language development using the average number of syllables per utterance.</t>
+          <t>The different types of sound it measured include:</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>La duración y variedad del habla de un niño mientras balbucea o habla con un adulto, lo que refleja el desarrollo del lenguaje utilizando el número promedio de sílabas por expresión.</t>
+          <t>Los diferentes tipos de sonido que midió incluyen:</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>The number of child vocalizations -or sounds- made by your child, including both words and "pre-word" sounds (like babbles, noises, and single sounds)</t>
+          <t>The length and variety of a child's speech while babbling or talking with an adult, reflecting language development using the average number of syllables per utterance.</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>La cantidad de vocalizaciones (o sonidos) infantiles que hace su hijo, incluidas tanto las palabras como los sonidos "prepalabras" (como balbuceos, ruidos y sonidos únicos)</t>
+          <t>La duración y variedad del habla de un niño mientras balbucea o habla con un adulto, lo que refleja el desarrollo del lenguaje utilizando el número promedio de sílabas por expresión.</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>These findings from the day of recording may not be accurate or representative of your child's everyday environment.</t>
+          <t>The number of child vocalizations -or sounds- made by your child, including both words and "pre-word" sounds (like babbles, noises, and single sounds)</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Es posible que estos hallazgos del día de la grabación no sean exactos o representativos del entorno cotidiano de su hijo.</t>
+          <t>La cantidad de vocalizaciones (o sonidos) infantiles que hace su hijo, incluidas tanto las palabras como los sonidos "prepalabras" (como balbuceos, ruidos y sonidos únicos)</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>This report contains</t>
+          <t>These findings from the day of recording may not be accurate or representative of your child's everyday environment.</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Este informe contiene</t>
+          <t>Es posible que estos hallazgos del día de la grabación no sean exactos o representativos del entorno cotidiano de su hijo.</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>This report describes the language and audio environment, which includes sounds, silence, speech, and other noises that the child can hear in the home environment of your child based on your LENA recording.</t>
+          <t>This report contains</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Este informe describe el entorno de lenguaje y audio, que incluye sonidos, silencio, habla y otros ruidos que el niño puede escuchar en el entorno hogareño de su hijo según su grabación LENA.</t>
+          <t>Este informe contiene</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>This report is based on a single day of recording, so it may not fully represent your family's typical language environment.</t>
+          <t>This report describes the language and audio environment, which includes sounds, silence, speech, and other noises that the child can hear in the home environment of your child based on your LENA recording.</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Este informe se basa en un solo día de grabación, por lo que es posible que no represente completamente el entorno lingüístico típico de su familia.</t>
+          <t>Este informe describe el entorno de lenguaje y audio, que incluye sonidos, silencio, habla y otros ruidos que el niño puede escuchar en el entorno hogareño de su hijo según su grabación LENA.</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>Total turns: 612</t>
+          <t>This report is based on a single day of recording, so it may not fully represent your family's typical language environment.</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Turnos totales: 612</t>
+          <t>Este informe se basa en un solo día de grabación, por lo que es posible que no represente completamente el entorno lingüístico típico de su familia.</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>Total turns: 845</t>
+          <t>Total turns: 612</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Turnos totales: 845</t>
+          <t>Turnos totales: 612</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>Total words/sounds: 2,210</t>
+          <t>Total turns: 845</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Total de palabras/sonidos: 2.210</t>
+          <t>Turnos totales: 845</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>Total words/sounds: 3,105</t>
+          <t>Total words/sounds: 2,210</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Total de palabras/sonidos: 3.105</t>
+          <t>Total de palabras/sonidos: 2.210</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>Touch, hug, hold</t>
+          <t>Total words/sounds: 3,105</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Tocar, abrazar, sostener</t>
+          <t>Total de palabras/sonidos: 3.105</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>Travis County Residents</t>
+          <t>Touch, hug, hold</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Residentes del condado de Travis</t>
+          <t>Tocar, abrazar, sostener</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>Tune in and respond</t>
+          <t>Travis County Residents</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Sintoniza y responde</t>
+          <t>Residentes del condado de Travis</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>UT Austin School of Nursing Wellness Centers</t>
+          <t>Tune in and respond</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Centros de bienestar de la Escuela de Enfermería de UT Austin</t>
+          <t>Sintoniza y responde</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>UT Austin School of Nursing provide health care services in two clinics: Children's Wellness Center (CWC) and Family Wellness Center (FWC), where nurse practitioners provide primary care and manage acute and chronic conditions.</t>
+          <t>UT Austin School of Nursing Wellness Centers</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>La Escuela de Enfermería de UT Austin brinda servicios de atención médica en dos clínicas: Children's Wellness Center (CWC) y Family Wellness Center (FWC), donde las enfermeras practicantes brindan atención primaria y manejan afecciones agudas y crónicas.</t>
+          <t>Centros de bienestar de la Escuela de Enfermería de UT Austin</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>Uninsured children in Central Texas</t>
+          <t>UT Austin School of Nursing provide health care services in two clinics: Children's Wellness Center (CWC) and Family Wellness Center (FWC), where nurse practitioners provide primary care and manage acute and chronic conditions.</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Niños sin seguro en el centro de Texas</t>
+          <t>La Escuela de Enfermería de UT Austin brinda servicios de atención médica en dos clínicas: Children's Wellness Center (CWC) y Family Wellness Center (FWC), donde las enfermeras practicantes brindan atención primaria y manejan afecciones agudas y crónicas.</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>United Way Family Resources</t>
+          <t>Uninsured children in Central Texas</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Recursos familiares de United Way</t>
+          <t>Niños sin seguro en el centro de Texas</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>United Way for Greater Austin focuses on increasing the availability of high-quality early care and education and access to pivotal resources to dismantle economic barriers in Central Texas.</t>
+          <t>United Way Family Resources</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>United Way for Greater Austin se enfoca en aumentar la disponibilidad de educación y cuidado infantil de alta calidad y el acceso a recursos fundamentales para desmantelar las barreras económicas en el centro de Texas.</t>
+          <t>Recursos familiares de United Way</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Vocal Productivity</t>
+          <t>United Way for Greater Austin focuses on increasing the availability of high-quality early care and education and access to pivotal resources to dismantle economic barriers in Central Texas.</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Productividad vocal</t>
+          <t>United Way for Greater Austin se enfoca en aumentar la disponibilidad de educación y cuidado infantil de alta calidad y el acceso a recursos fundamentales para desmantelar las barreras económicas en el centro de Texas.</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>WCWH uses the database to compare your child's recording to recordings in the database to identify your child's percentiles.</t>
+          <t>Vocal Productivity</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>WCWH utiliza la base de datos para comparar los registros de su hijo con los registros de la base de datos para identificar los percentiles de su hijo.</t>
+          <t>Productividad vocal</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>Wait for their response</t>
+          <t>WCWH uses the database to compare your child's recording to recordings in the database to identify your child's percentiles.</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Espere su respuesta</t>
+          <t>WCWH utiliza la base de datos para comparar los registros de su hijo con los registros de la base de datos para identificar los percentiles de su hijo.</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>Ways you can do to support your child's language growth, improving their vocabulary/reading skills, brain structure/function, assessment scores, and social-emotional development.</t>
+          <t>Wait for their response</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Formas que puede hacer para apoyar el crecimiento del lenguaje de su hijo, mejorar su vocabulario/habilidades de lectura, estructura/función cerebral, puntajes de evaluación y desarrollo socioemocional.</t>
+          <t>Espere su respuesta</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>We understand it can be tricky to get a full 24-hour recording. Remember to reach out to our study staff to troubleshoot with LENA use-and-wear. If you want to try again, please contact us to schedule another LENA drop-off.</t>
+          <t>Ways you can do to support your child's language growth, improving their vocabulary/reading skills, brain structure/function, assessment scores, and social-emotional development.</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Entendemos que puede resultar complicado obtener una grabación completa de 24 horas. Recuerde comunicarse con nuestro personal del estudio para solucionar problemas con el uso y uso de LENA. Si desea volver a intentarlo, comuníquese con nosotros para programar otra entrega de LENA.</t>
+          <t>Formas que puede hacer para apoyar el crecimiento del lenguaje de su hijo, mejorar su vocabulario/habilidades de lectura, estructura/función cerebral, puntajes de evaluación y desarrollo socioemocional.</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>What is LENA Database</t>
+          <t>We understand it can be tricky to get a full 24-hour recording. Remember to reach out to our study staff to troubleshoot with LENA use-and-wear. If you want to try again, please contact us to schedule another LENA drop-off.</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>¿Qué es la base de datos LENA?</t>
+          <t>Entendemos que puede resultar complicado obtener una grabación completa de 24 horas. Recuerde comunicarse con nuestro personal del estudio para solucionar problemas con el uso y uso de LENA. Si desea volver a intentarlo, comuníquese con nosotros para programar otra entrega de LENA.</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>When a child and an adult talk together, going back-and-forth in the conversation.</t>
+          <t>What is LENA Database</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Cuando un niño y un adulto hablan juntos, van y vienen en la conversación.</t>
+          <t>¿Qué es la base de datos LENA?</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Whose Data is Included</t>
+          <t>When a child and an adult talk together, going back-and-forth in the conversation.</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Cuyos datos están incluidos</t>
+          <t>Cuando un niño y un adulto hablan juntos, van y vienen en la conversación.</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>You can click on any links and catalogs in this report. They will take you to websites or other pages in the report.</t>
+          <t>Whose Data is Included</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Puede hacer clic en cualquier enlace y catálogo de este informe. Lo llevarán a sitios web u otras páginas del informe.</t>
+          <t>Cuyos datos están incluidos</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Young children and families</t>
+          <t>You can click on any links and catalogs in this report. They will take you to websites or other pages in the report.</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Niños pequeños y familias</t>
+          <t>Puede hacer clic en cualquier enlace y catálogo de este informe. Lo llevarán a sitios web u otras páginas del informe.</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Your child has about the same number of conversational turns as most children their age.</t>
+          <t>Young children and families</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Su hijo tiene aproximadamente la misma cantidad de turnos de conversación que la mayoría de los niños de su edad.</t>
+          <t>Niños pequeños y familias</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>Your child has more conversational turns than most children their age.</t>
+          <t>Your child has about the same number of conversational turns as most children their age.</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Su hijo tiene más turnos de conversación que la mayoría de los niños de su edad.</t>
+          <t>Su hijo tiene aproximadamente la misma cantidad de turnos de conversación que la mayoría de los niños de su edad.</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>Your child uses more utterances within conversations than most children their age.</t>
+          <t>Your child has more conversational turns than most children their age.</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Su hijo utiliza más expresiones en las conversaciones que la mayoría de los niños de su edad.</t>
+          <t>Su hijo tiene más turnos de conversación que la mayoría de los niños de su edad.</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>Your child vocalizes more than most children their age.</t>
+          <t>Your child uses more utterances within conversations than most children their age.</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Su hijo vocaliza más que la mayoría de los niños de su edad.</t>
+          <t>Su hijo utiliza más expresiones en las conversaciones que la mayoría de los niños de su edad.</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Your child's utterances within conversations are about the same as most children their age.</t>
+          <t>Your child vocalizes more than most children their age.</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Las expresiones de su hijo durante las conversaciones son aproximadamente las mismas que las de la mayoría de los niños de su edad.</t>
+          <t>Su hijo vocaliza más que la mayoría de los niños de su edad.</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>about how your LENA recording compares to LENA recordings from other children and households that may or may not be like your own.</t>
+          <t>Your child's utterances within conversations are about the same as most children their age.</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>sobre cómo se compara su grabación LENA con las grabaciones LENA de otros niños y hogares que pueden o no ser como el suyo.</t>
+          <t>Las expresiones de su hijo durante las conversaciones son aproximadamente las mismas que las de la mayoría de los niños de su edad.</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>ask@b3tx.org</t>
+          <t>about how your LENA recording compares to LENA recordings from other children and households that may or may not be like your own.</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>pregunte@b3tx.org</t>
+          <t>sobre cómo se compara su grabación LENA con las grabaciones LENA de otros niños y hogares que pueden o no ser como el suyo.</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>bastropfamilyconnects@lscctx.org</t>
+          <t>ask@b3tx.org</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>bastropfamilyconnects@lscctx.org</t>
+          <t>pregunte@b3tx.org</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>contact@mylantern.org</t>
+          <t>bastropfamilyconnects@lscctx.org</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>contacto@mylantern.org</t>
+          <t>bastropfamilyconnects@lscctx.org</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>customercare@chcsct.com</t>
+          <t>contact@mylantern.org</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>atención al cliente@chcsct.com</t>
+          <t>contacto@mylantern.org</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>info@anybabycan.org</t>
+          <t>customercare@chcsct.com</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>info@anybabycan.org</t>
+          <t>atención al cliente@chcsct.com</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>info@bookspring.org</t>
+          <t>info@anybabycan.org</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>info@bookspring.org</t>
+          <t>info@anybabycan.org</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>info@bookspring.org</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>información</t>
+          <t>info@bookspring.org</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>on their words</t>
+          <t>information</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>en sus palabras</t>
+          <t>información</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>that interest them</t>
+          <t>on their words</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>que les interese</t>
+          <t>en sus palabras</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>to what they notice</t>
+          <t>that interest them</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>a lo que notan</t>
+          <t>que les interese</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>utsoncwc@nursing.utexas.edu</t>
+          <t>to what they notice</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>utsoncwc@nursing.utexas.edu</t>
+          <t>a lo que notan</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>wcwhcommunity@austin.utexas.edu</t>
+          <t>utsoncwc@nursing.utexas.edu</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>wcwhcommunity@austin.utexas.edu</t>
+          <t>utsoncwc@nursing.utexas.edu</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>what they see or do</t>
+          <t>wcwhcommunity@austin.utexas.edu</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>lo que ven o hacen</t>
+          <t>wcwhcommunity@austin.utexas.edu</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>what you're doing</t>
+          <t>what they see or do</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>que estas haciendo</t>
+          <t>lo que ven o hacen</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>what you're doing</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>|</t>
+          <t>que estas haciendo</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
+          <t>|</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>|</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
           <t>– don't do all the talking</t>
         </is>
       </c>
-      <c r="B265" t="inlineStr">
+      <c r="B266" t="inlineStr">
         <is>
           <t>– no hables solo</t>
         </is>

</xml_diff>